<commit_message>
Update INARA 2026-09-13 18:12:46
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1552,7 +1552,7 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16" t="b">
         <v>1</v>
@@ -1605,10 +1605,10 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="s">
         <v>114</v>
@@ -1658,10 +1658,10 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="s">
         <v>114</v>
@@ -1976,10 +1976,10 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q24" t="s">
         <v>114</v>
@@ -2029,10 +2029,10 @@
         <v>0</v>
       </c>
       <c r="O25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q25" t="s">
         <v>114</v>
@@ -2082,10 +2082,10 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q26" t="s">
         <v>114</v>
@@ -2135,10 +2135,10 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="s">
         <v>114</v>
@@ -2600,7 +2600,7 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P36" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-14 20:51:19
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1905,10 +1905,10 @@
         <v>101</v>
       </c>
       <c r="I23">
-        <v>-8.589625893999999</v>
+        <v>0</v>
       </c>
       <c r="J23">
-        <v>116.3057965</v>
+        <v>0</v>
       </c>
       <c r="K23" t="s">
         <v>112</v>
@@ -2682,22 +2682,22 @@
         <v>109</v>
       </c>
       <c r="I38">
-        <v>-8.364740604</v>
+        <v>0</v>
       </c>
       <c r="J38">
-        <v>115.1918556</v>
+        <v>0</v>
       </c>
       <c r="K38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M38">
         <v>0</v>
       </c>
       <c r="N38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O38">
         <v>5</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-15 10:25:35
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -2600,7 +2600,7 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P36" t="b">
         <v>1</v>
@@ -2650,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P37" t="b">
         <v>1</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="O38">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P38" t="b">
         <v>1</v>
@@ -2750,7 +2750,7 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P39" t="b">
         <v>1</v>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P40" t="b">
         <v>1</v>
@@ -2850,7 +2850,7 @@
         <v>1</v>
       </c>
       <c r="O41">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="P41" t="b">
         <v>1</v>
@@ -2900,7 +2900,7 @@
         <v>1</v>
       </c>
       <c r="O42">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="P42" t="b">
         <v>1</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P43" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-16 11:59:12
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1234,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P10" t="b">
         <v>1</v>
@@ -1287,7 +1287,7 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P11" t="b">
         <v>1</v>
@@ -1340,7 +1340,7 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P12" t="b">
         <v>1</v>
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P13" t="b">
         <v>1</v>
@@ -1976,7 +1976,7 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P24" t="b">
         <v>1</v>
@@ -2347,10 +2347,10 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31" t="s">
         <v>114</v>
@@ -2600,7 +2600,7 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P36" t="b">
         <v>1</v>
@@ -2650,7 +2650,7 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P37" t="b">
         <v>1</v>
@@ -2700,7 +2700,7 @@
         <v>1</v>
       </c>
       <c r="O38">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="P38" t="b">
         <v>1</v>
@@ -2750,7 +2750,7 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P39" t="b">
         <v>1</v>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P40" t="b">
         <v>1</v>
@@ -2850,7 +2850,7 @@
         <v>1</v>
       </c>
       <c r="O41">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P41" t="b">
         <v>1</v>
@@ -2900,7 +2900,7 @@
         <v>1</v>
       </c>
       <c r="O42">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P42" t="b">
         <v>1</v>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="O43">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="P43" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-17 11:38:56
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -795,10 +795,10 @@
         <v>93</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>-8.508568474</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>115.1998034</v>
       </c>
       <c r="K2" t="s">
         <v>111</v>
@@ -898,10 +898,10 @@
         <v>95</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>-8.602909052999999</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>116.1536542</v>
       </c>
       <c r="K4" t="s">
         <v>111</v>
@@ -1163,10 +1163,10 @@
         <v>98</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>-8.627538016000001</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>116.1327942</v>
       </c>
       <c r="K9" t="s">
         <v>112</v>
@@ -1269,10 +1269,10 @@
         <v>99</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>-8.358866183</v>
       </c>
       <c r="J11">
-        <v>0</v>
+        <v>116.1487853</v>
       </c>
       <c r="K11" t="s">
         <v>112</v>
@@ -1375,10 +1375,10 @@
         <v>100</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>-8.347617261</v>
       </c>
       <c r="J13">
-        <v>0</v>
+        <v>116.1690833</v>
       </c>
       <c r="K13" t="s">
         <v>111</v>
@@ -1905,10 +1905,10 @@
         <v>101</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>-8.589625893999999</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>116.3057965</v>
       </c>
       <c r="K23" t="s">
         <v>112</v>
@@ -2011,10 +2011,10 @@
         <v>102</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>-8.587743615999999</v>
       </c>
       <c r="J25">
-        <v>0</v>
+        <v>116.3199546</v>
       </c>
       <c r="K25" t="s">
         <v>113</v>
@@ -2170,10 +2170,10 @@
         <v>104</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>-8.592968228</v>
       </c>
       <c r="J28">
-        <v>0</v>
+        <v>116.2928783</v>
       </c>
       <c r="K28" t="s">
         <v>111</v>
@@ -2329,10 +2329,10 @@
         <v>102</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>-8.801802138999999</v>
       </c>
       <c r="J31">
-        <v>0</v>
+        <v>116.23624</v>
       </c>
       <c r="K31" t="s">
         <v>112</v>
@@ -2432,10 +2432,10 @@
         <v>107</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>-10.15818294</v>
       </c>
       <c r="J33">
-        <v>0</v>
+        <v>123.6654479</v>
       </c>
       <c r="K33" t="s">
         <v>113</v>
@@ -2532,10 +2532,10 @@
         <v>108</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>-8.699028999999999</v>
       </c>
       <c r="J35">
-        <v>0</v>
+        <v>115.2086979</v>
       </c>
       <c r="K35" t="s">
         <v>111</v>
@@ -2582,10 +2582,10 @@
         <v>109</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>-8.369822170999999</v>
       </c>
       <c r="J36">
-        <v>0</v>
+        <v>115.1925405</v>
       </c>
       <c r="K36" t="s">
         <v>113</v>
@@ -2682,10 +2682,10 @@
         <v>109</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>-8.364740604</v>
       </c>
       <c r="J38">
-        <v>0</v>
+        <v>115.1918556</v>
       </c>
       <c r="K38" t="s">
         <v>111</v>
@@ -2738,16 +2738,16 @@
         <v>115.1953139</v>
       </c>
       <c r="K39" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M39">
         <v>1</v>
       </c>
       <c r="N39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O39">
         <v>10</v>
@@ -2832,10 +2832,10 @@
         <v>110</v>
       </c>
       <c r="I41">
-        <v>0</v>
+        <v>-8.394319465000001</v>
       </c>
       <c r="J41">
-        <v>0</v>
+        <v>115.1955146</v>
       </c>
       <c r="K41" t="s">
         <v>111</v>
@@ -2882,10 +2882,10 @@
         <v>110</v>
       </c>
       <c r="I42">
-        <v>0</v>
+        <v>-8.401367157999999</v>
       </c>
       <c r="J42">
-        <v>0</v>
+        <v>115.1964986</v>
       </c>
       <c r="K42" t="s">
         <v>113</v>
@@ -2938,16 +2938,16 @@
         <v>115.1969283</v>
       </c>
       <c r="K43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M43">
         <v>0</v>
       </c>
       <c r="N43">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O43">
         <v>10</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-20 09:26:13
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1022,7 +1022,7 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P6" t="b">
         <v>1</v>
@@ -1976,7 +1976,7 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P24" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-21 16:24:01
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -2638,16 +2638,16 @@
         <v>115.1921949</v>
       </c>
       <c r="K37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M37">
         <v>0</v>
       </c>
       <c r="N37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O37">
         <v>10</v>
@@ -2741,13 +2741,13 @@
         <v>113</v>
       </c>
       <c r="L39">
+        <v>3</v>
+      </c>
+      <c r="M39">
+        <v>1</v>
+      </c>
+      <c r="N39">
         <v>2</v>
-      </c>
-      <c r="M39">
-        <v>1</v>
-      </c>
-      <c r="N39">
-        <v>1</v>
       </c>
       <c r="O39">
         <v>10</v>
@@ -2891,13 +2891,13 @@
         <v>113</v>
       </c>
       <c r="L42">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M42">
         <v>2</v>
       </c>
       <c r="N42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O42">
         <v>11</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-23 15:57:56
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -2688,16 +2688,16 @@
         <v>115.1918556</v>
       </c>
       <c r="K38" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="L38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M38">
         <v>0</v>
       </c>
       <c r="N38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O38">
         <v>10</v>
@@ -2891,13 +2891,13 @@
         <v>113</v>
       </c>
       <c r="L42">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M42">
         <v>2</v>
       </c>
       <c r="N42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O42">
         <v>11</v>
@@ -2938,7 +2938,7 @@
         <v>115.1969283</v>
       </c>
       <c r="K43" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L43">
         <v>2</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-24 10:01:18
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1905,10 +1905,10 @@
         <v>101</v>
       </c>
       <c r="I23">
-        <v>-8.589625893999999</v>
+        <v>-8.589509</v>
       </c>
       <c r="J23">
-        <v>116.3057965</v>
+        <v>116.3057</v>
       </c>
       <c r="K23" t="s">
         <v>112</v>
@@ -2438,7 +2438,7 @@
         <v>123.6654479</v>
       </c>
       <c r="K33" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L33">
         <v>2</v>
@@ -2588,7 +2588,7 @@
         <v>115.1925405</v>
       </c>
       <c r="K36" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L36">
         <v>2</v>
@@ -2688,7 +2688,7 @@
         <v>115.1918556</v>
       </c>
       <c r="K38" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L38">
         <v>2</v>
@@ -2738,16 +2738,16 @@
         <v>115.1953139</v>
       </c>
       <c r="K39" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M39">
         <v>1</v>
       </c>
       <c r="N39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O39">
         <v>10</v>
@@ -2941,13 +2941,13 @@
         <v>111</v>
       </c>
       <c r="L43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M43">
         <v>0</v>
       </c>
       <c r="N43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O43">
         <v>10</v>

</xml_diff>

<commit_message>
Update INARA 2026-09-28 13:09:39
</commit_message>
<xml_diff>
--- a/detail_odp_black_special_value.xlsx
+++ b/detail_odp_black_special_value.xlsx
@@ -1911,16 +1911,16 @@
         <v>116.3057</v>
       </c>
       <c r="K23" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23">
         <v>2</v>

</xml_diff>